<commit_message>
fix names df names in the build_df function
</commit_message>
<xml_diff>
--- a/itens.xlsx
+++ b/itens.xlsx
@@ -419,17 +419,17 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>nome</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>price</t>
+          <t>preco</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>book_url</t>
+          <t>url</t>
         </is>
       </c>
     </row>

</xml_diff>